<commit_message>
Osijek, Zadar, Varaždin (API) i Bjelovar, Orahovica, Drenovci, Belišće, Čazma, Grubišno Polje, Ilok, općine oko Vukovara
- Osijek (Unikom, 9 JLS, 74 zone), Zadar (Čistoća Zadar, 19 JLS uključujući
  Sveti Filip i Jakov, 90 zona) i Varaždin (Čistoća Varaždin, grad i 11
  općina, 31 zona): javni API-ji po adresi, istovjetni rasporedi spojeni u
  zone; usporedba s ispisom rasporeda davatelja za uzorak adresa (Zadar
  dodatno provjeren uživo: 0 razlika).
- Komunalac Bjelovar (grad i 8 općina, 35 zona); dani miješanog otpada za
  općine iz obavijesti (dio iz 2025., navedeno u napomeni).
- Papuk, Drenovci, Kombel, Komunalije Čazma, Komunalac Grubišno Polje,
  Kom-Ilok (pravila iz 2025.).
- Komunalac Vukovar: dodane općine Bogdanovci, Negoslavci i Tompojevci;
  zone grada nepromijenjene.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012grr9UJafq4ZimrFiB6wUv
</commit_message>
<xml_diff>
--- a/excel/vukovar-komunalac/Pregled_zona.xlsx
+++ b/excel/vukovar-komunalac/Pregled_zona.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1003,6 +1003,117 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Bogdanovci</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Općina Bogdanovci (ponedjeljak): Bogdanovci, Petrovci, Svinjarevci</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>ponedjeljak</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Miješani komunalni otpad, Biootpad, Plastika i metal, Papir i karton, Staklena ambalaža, Glomazni otpad</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>2026: 92</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Bogdanovci, Petrovci, Svinjarevci</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Tompojevci</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Općina Tompojevci (petak, svaki drugi tjedan): Berak, Čakovci, Bokšić, Tompojevci, Mikluševci</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>petak</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Miješani komunalni otpad, Biootpad, Plastika i metal, Papir i karton, Staklena ambalaža, Glomazni otpad</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>2026: 80</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Berak, Čakovci, Bokšić, Tompojevci, Mikluševci</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Negoslavci</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Općina Negoslavci (srijeda): Negoslavci</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>srijeda</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Miješani komunalni otpad, Biootpad, Plastika i metal, Papir i karton, Staklena ambalaža, Glomazni otpad</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>2026: 107</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Negoslavci</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>